<commit_message>
updated as a clean lib
</commit_message>
<xml_diff>
--- a/doc/design/design.xlsx
+++ b/doc/design/design.xlsx
@@ -1,35 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects.git\esp32_remote_control\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects.git\esp32_remote_control\doc\design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776CD1C7-AE44-4AF9-9E60-1E16F87ED6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B9EDA9-ED83-4754-8257-AF9BF357CC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="69012" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="527" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" tabRatio="527" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="2" r:id="rId1"/>
-    <sheet name="ESP32 PIN Design" sheetId="1" r:id="rId2"/>
-    <sheet name="NRF24L01" sheetId="4" r:id="rId3"/>
-    <sheet name="ESP32 38 PINS" sheetId="3" r:id="rId4"/>
-    <sheet name="ICM 90248" sheetId="5" r:id="rId5"/>
+    <sheet name="ESP32 Dev Design" sheetId="1" r:id="rId2"/>
+    <sheet name="ESP32-S3 Design" sheetId="7" r:id="rId3"/>
+    <sheet name="NRF24L01" sheetId="4" r:id="rId4"/>
+    <sheet name="ESP32 38 PINS" sheetId="3" r:id="rId5"/>
+    <sheet name="ESP32 S3" sheetId="6" r:id="rId6"/>
+    <sheet name="ICM 90248" sheetId="5" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="164">
   <si>
     <t>Main Controller</t>
   </si>
@@ -459,6 +475,74 @@
   </si>
   <si>
     <t>HSPI CSN</t>
+  </si>
+  <si>
+    <t>ESP32 S3 Pin Suggestion</t>
+  </si>
+  <si>
+    <t>Pot1 (Analog Signal)</t>
+  </si>
+  <si>
+    <t>Pot2 (Analog Signal)</t>
+  </si>
+  <si>
+    <t>Potentiometer (2x)</t>
+  </si>
+  <si>
+    <t>Power Switch</t>
+  </si>
+  <si>
+    <t>RGB LED (w2812b)</t>
+  </si>
+  <si>
+    <t>3 x 18650 battery (dual voltage input)</t>
+  </si>
+  <si>
+    <t>Lock Switch (2x)</t>
+  </si>
+  <si>
+    <t>Power LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiny LED </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each LED can show different color, blink for different state.
+</t>
+  </si>
+  <si>
+    <t>1 - External Antena 
+2 - Power socket adapter</t>
+  </si>
+  <si>
+    <t>Color Buttons (4x)</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>Shared by TFT, MPU, NRF24L01</t>
+  </si>
+  <si>
+    <t>GPIO39</t>
+  </si>
+  <si>
+    <t>GPIO40</t>
+  </si>
+  <si>
+    <t>GPIO41</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>RF SPI clock</t>
+  </si>
+  <si>
+    <t>RF SPI MISO</t>
+  </si>
+  <si>
+    <t>RF SPI MOSI</t>
   </si>
 </sst>
 </file>
@@ -516,7 +600,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -604,8 +688,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -694,6 +784,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -701,7 +828,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -815,6 +942,30 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -830,29 +981,42 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1137,16 +1301,82 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>566737</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>452437</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{779858A2-2A9E-F6A6-64A5-3A4A274EFCE4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1214437" y="381000"/>
+          <a:ext cx="12192000" cy="8334375"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>433388</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>23813</xdr:rowOff>
+      <xdr:colOff>429725</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>122727</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>331498</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>23843</xdr:rowOff>
+      <xdr:colOff>327835</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>122757</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1169,8 +1399,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="432436" y="205741"/>
-          <a:ext cx="3555710" cy="3840510"/>
+          <a:off x="429725" y="122727"/>
+          <a:ext cx="3788706" cy="3769732"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1182,15 +1412,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>391987</xdr:colOff>
+      <xdr:colOff>289410</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>146538</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>480590</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>96084</xdr:rowOff>
+      <xdr:colOff>378013</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>63112</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1213,8 +1443,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4661092" y="0"/>
-          <a:ext cx="1917403" cy="3022164"/>
+          <a:off x="4828439" y="146538"/>
+          <a:ext cx="2033901" cy="2968238"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1490,15 +1720,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{065EAA11-B65B-4544-88B3-3334179E6B90}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="27.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.77734375" customWidth="1"/>
-    <col min="5" max="5" width="14.21875" customWidth="1"/>
-    <col min="6" max="6" width="28.21875" customWidth="1"/>
+    <col min="2" max="2" width="27.1328125" customWidth="1"/>
+    <col min="3" max="3" width="38.796875" customWidth="1"/>
+    <col min="5" max="5" width="14.19921875" customWidth="1"/>
+    <col min="6" max="6" width="28.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>18</v>
@@ -1513,7 +1743,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1527,7 +1757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1541,7 +1771,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1558,7 +1788,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1572,7 +1802,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1586,7 +1816,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1597,7 +1827,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1611,7 +1841,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1625,7 +1855,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1639,7 +1869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1653,7 +1883,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1678,17 +1908,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F68"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" style="13" customWidth="1"/>
-    <col min="4" max="4" width="24.88671875" style="13" customWidth="1"/>
-    <col min="5" max="5" width="33.21875" customWidth="1"/>
-    <col min="6" max="6" width="33.44140625" customWidth="1"/>
+    <col min="3" max="3" width="21.46484375" style="13" customWidth="1"/>
+    <col min="4" max="4" width="24.86328125" style="13" customWidth="1"/>
+    <col min="5" max="5" width="33.19921875" customWidth="1"/>
+    <col min="6" max="6" width="33.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="16" t="s">
         <v>24</v>
       </c>
@@ -1708,8 +1938,8 @@
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="53" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" s="43" t="s">
         <v>115</v>
       </c>
       <c r="B2" s="17" t="s">
@@ -1726,8 +1956,8 @@
       </c>
       <c r="F2" s="36"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="53"/>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3" s="43"/>
       <c r="B3" s="17" t="s">
         <v>108</v>
       </c>
@@ -1742,8 +1972,8 @@
       </c>
       <c r="F3" s="36"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="53"/>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="43"/>
       <c r="B4" s="17" t="s">
         <v>109</v>
       </c>
@@ -1758,8 +1988,8 @@
       </c>
       <c r="F4" s="36"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="53"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5" s="43"/>
       <c r="B5" s="37" t="s">
         <v>30</v>
       </c>
@@ -1774,8 +2004,8 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="53"/>
+    <row r="6" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="43"/>
       <c r="B6" s="17" t="s">
         <v>110</v>
       </c>
@@ -1788,8 +2018,8 @@
       <c r="E6" s="17"/>
       <c r="F6" s="36"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="49" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7" s="42" t="s">
         <v>116</v>
       </c>
       <c r="B7" s="18" t="s">
@@ -1806,8 +2036,8 @@
       </c>
       <c r="F7" s="36"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="49"/>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" s="42"/>
       <c r="B8" s="18" t="s">
         <v>125</v>
       </c>
@@ -1822,8 +2052,8 @@
       </c>
       <c r="F8" s="36"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="49"/>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A9" s="42"/>
       <c r="B9" s="18" t="s">
         <v>126</v>
       </c>
@@ -1838,8 +2068,8 @@
       </c>
       <c r="F9" s="36"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="49"/>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" s="42"/>
       <c r="B10" s="18" t="s">
         <v>127</v>
       </c>
@@ -1854,8 +2084,8 @@
       </c>
       <c r="F10" s="36"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="49"/>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11" s="42"/>
       <c r="B11" s="18" t="s">
         <v>33</v>
       </c>
@@ -1868,8 +2098,8 @@
       </c>
       <c r="F11" s="36"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="52" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12" s="47" t="s">
         <v>117</v>
       </c>
       <c r="B12" s="19" t="s">
@@ -1886,8 +2116,8 @@
       </c>
       <c r="F12" s="36"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="52"/>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13" s="47"/>
       <c r="B13" s="19" t="s">
         <v>112</v>
       </c>
@@ -1902,8 +2132,8 @@
       </c>
       <c r="F13" s="36"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="52"/>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14" s="47"/>
       <c r="B14" s="19" t="s">
         <v>113</v>
       </c>
@@ -1918,8 +2148,8 @@
       </c>
       <c r="F14" s="36"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="52"/>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15" s="47"/>
       <c r="B15" s="19" t="s">
         <v>141</v>
       </c>
@@ -1934,8 +2164,8 @@
       </c>
       <c r="F15" s="36"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="52"/>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16" s="47"/>
       <c r="B16" s="19" t="s">
         <v>37</v>
       </c>
@@ -1950,7 +2180,7 @@
       </c>
       <c r="F16" s="36"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" s="40" t="s">
         <v>2</v>
       </c>
@@ -1968,8 +2198,8 @@
       </c>
       <c r="F17" s="35"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="49" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18" s="42" t="s">
         <v>40</v>
       </c>
       <c r="B18" s="18" t="s">
@@ -1986,8 +2216,8 @@
       </c>
       <c r="F18" s="35"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="49"/>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" s="42"/>
       <c r="B19" s="18" t="s">
         <v>43</v>
       </c>
@@ -2002,8 +2232,8 @@
       </c>
       <c r="F19" s="35"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="49"/>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20" s="42"/>
       <c r="B20" s="18" t="s">
         <v>44</v>
       </c>
@@ -2018,8 +2248,8 @@
       </c>
       <c r="F20" s="35"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="49"/>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21" s="42"/>
       <c r="B21" s="18" t="s">
         <v>45</v>
       </c>
@@ -2034,8 +2264,8 @@
       </c>
       <c r="F21" s="35"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="42" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22" s="50" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="21" t="s">
@@ -2050,8 +2280,8 @@
       <c r="E22" s="21"/>
       <c r="F22" s="35"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="43"/>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23" s="51"/>
       <c r="B23" s="21" t="s">
         <v>48</v>
       </c>
@@ -2064,7 +2294,7 @@
       <c r="E23" s="21"/>
       <c r="F23" s="35"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" s="22" t="s">
         <v>10</v>
       </c>
@@ -2082,8 +2312,8 @@
       </c>
       <c r="F24" s="35"/>
     </row>
-    <row r="25" spans="1:6" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="44" t="s">
+    <row r="25" spans="1:6" ht="25.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="52" t="s">
         <v>49</v>
       </c>
       <c r="B25" s="24" t="s">
@@ -2098,8 +2328,8 @@
       <c r="E25" s="24"/>
       <c r="F25" s="35"/>
     </row>
-    <row r="26" spans="1:6" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="45"/>
+    <row r="26" spans="1:6" ht="25.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="53"/>
       <c r="B26" s="24" t="s">
         <v>50</v>
       </c>
@@ -2112,8 +2342,8 @@
       <c r="E26" s="24"/>
       <c r="F26" s="35"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="49" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A27" s="42" t="s">
         <v>51</v>
       </c>
       <c r="B27" s="18" t="s">
@@ -2128,8 +2358,8 @@
       <c r="E27" s="18"/>
       <c r="F27" s="35"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="49"/>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A28" s="42"/>
       <c r="B28" s="18" t="s">
         <v>53</v>
       </c>
@@ -2142,8 +2372,8 @@
       <c r="E28" s="18"/>
       <c r="F28" s="35"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="49"/>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A29" s="42"/>
       <c r="B29" s="18" t="s">
         <v>54</v>
       </c>
@@ -2156,8 +2386,8 @@
       <c r="E29" s="18"/>
       <c r="F29" s="35"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="49"/>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A30" s="42"/>
       <c r="B30" s="18" t="s">
         <v>55</v>
       </c>
@@ -2170,8 +2400,8 @@
       <c r="E30" s="18"/>
       <c r="F30" s="35"/>
     </row>
-    <row r="35" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="36" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="36" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A36" s="14" t="s">
         <v>56</v>
       </c>
@@ -2186,7 +2416,7 @@
       </c>
       <c r="E36" s="32"/>
     </row>
-    <row r="37" spans="1:5" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="37" spans="1:5" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="1.05">
       <c r="A37" s="2" t="s">
         <v>60</v>
       </c>
@@ -2196,12 +2426,12 @@
       <c r="C37" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="50" t="s">
+      <c r="D37" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="50"/>
-    </row>
-    <row r="38" spans="1:5" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E37" s="44"/>
+    </row>
+    <row r="38" spans="1:5" ht="29.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A38" s="4" t="s">
         <v>63</v>
       </c>
@@ -2211,12 +2441,12 @@
       <c r="C38" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="47" t="s">
+      <c r="D38" s="45" t="s">
         <v>65</v>
       </c>
-      <c r="E38" s="47"/>
-    </row>
-    <row r="39" spans="1:5" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E38" s="45"/>
+    </row>
+    <row r="39" spans="1:5" ht="43.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A39" s="6" t="s">
         <v>66</v>
       </c>
@@ -2226,12 +2456,12 @@
       <c r="C39" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D39" s="51" t="s">
+      <c r="D39" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="E39" s="51"/>
-    </row>
-    <row r="40" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E39" s="46"/>
+    </row>
+    <row r="40" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A40" s="4" t="s">
         <v>68</v>
       </c>
@@ -2241,12 +2471,12 @@
       <c r="C40" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D40" s="47" t="s">
+      <c r="D40" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="E40" s="47"/>
-    </row>
-    <row r="41" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E40" s="45"/>
+    </row>
+    <row r="41" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A41" s="8" t="s">
         <v>70</v>
       </c>
@@ -2256,10 +2486,10 @@
       <c r="C41" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D41" s="41"/>
-      <c r="E41" s="41"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D41" s="49"/>
+      <c r="E41" s="49"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" s="11" t="s">
         <v>72</v>
       </c>
@@ -2269,12 +2499,12 @@
       <c r="C42" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D42" s="46" t="s">
+      <c r="D42" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="E42" s="46"/>
-    </row>
-    <row r="43" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E42" s="48"/>
+    </row>
+    <row r="43" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A43" s="4" t="s">
         <v>74</v>
       </c>
@@ -2284,12 +2514,12 @@
       <c r="C43" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="47" t="s">
+      <c r="D43" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="E43" s="47"/>
-    </row>
-    <row r="44" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E43" s="45"/>
+    </row>
+    <row r="44" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A44" s="4" t="s">
         <v>76</v>
       </c>
@@ -2299,12 +2529,12 @@
       <c r="C44" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D44" s="47" t="s">
+      <c r="D44" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="E44" s="47"/>
-    </row>
-    <row r="45" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E44" s="45"/>
+    </row>
+    <row r="45" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A45" s="4" t="s">
         <v>77</v>
       </c>
@@ -2314,12 +2544,12 @@
       <c r="C45" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D45" s="47" t="s">
+      <c r="D45" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="E45" s="47"/>
-    </row>
-    <row r="46" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E45" s="45"/>
+    </row>
+    <row r="46" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A46" s="4" t="s">
         <v>78</v>
       </c>
@@ -2329,12 +2559,12 @@
       <c r="C46" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="47" t="s">
+      <c r="D46" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="E46" s="47"/>
-    </row>
-    <row r="47" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E46" s="45"/>
+    </row>
+    <row r="47" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A47" s="4" t="s">
         <v>79</v>
       </c>
@@ -2344,12 +2574,12 @@
       <c r="C47" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D47" s="47" t="s">
+      <c r="D47" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="E47" s="47"/>
-    </row>
-    <row r="48" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E47" s="45"/>
+    </row>
+    <row r="48" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A48" s="4" t="s">
         <v>80</v>
       </c>
@@ -2359,12 +2589,12 @@
       <c r="C48" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="47" t="s">
+      <c r="D48" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="E48" s="47"/>
-    </row>
-    <row r="49" spans="1:5" ht="78" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E48" s="45"/>
+    </row>
+    <row r="49" spans="1:5" ht="78" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A49" s="11" t="s">
         <v>81</v>
       </c>
@@ -2374,12 +2604,12 @@
       <c r="C49" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D49" s="46" t="s">
+      <c r="D49" s="48" t="s">
         <v>119</v>
       </c>
-      <c r="E49" s="46"/>
-    </row>
-    <row r="50" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E49" s="48"/>
+    </row>
+    <row r="50" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A50" s="8" t="s">
         <v>82</v>
       </c>
@@ -2392,7 +2622,7 @@
       <c r="D50" s="33"/>
       <c r="E50" s="10"/>
     </row>
-    <row r="51" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
@@ -2405,7 +2635,7 @@
       <c r="D51" s="33"/>
       <c r="E51" s="10"/>
     </row>
-    <row r="52" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A52" s="11" t="s">
         <v>84</v>
       </c>
@@ -2415,12 +2645,12 @@
       <c r="C52" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D52" s="48" t="s">
+      <c r="D52" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="E52" s="48"/>
-    </row>
-    <row r="53" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E52" s="54"/>
+    </row>
+    <row r="53" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A53" s="8" t="s">
         <v>86</v>
       </c>
@@ -2430,10 +2660,10 @@
       <c r="C53" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D53" s="41"/>
-      <c r="E53" s="41"/>
-    </row>
-    <row r="54" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D53" s="49"/>
+      <c r="E53" s="49"/>
+    </row>
+    <row r="54" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A54" s="8" t="s">
         <v>87</v>
       </c>
@@ -2443,10 +2673,10 @@
       <c r="C54" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D54" s="41"/>
-      <c r="E54" s="41"/>
-    </row>
-    <row r="55" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D54" s="49"/>
+      <c r="E54" s="49"/>
+    </row>
+    <row r="55" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A55" s="8" t="s">
         <v>88</v>
       </c>
@@ -2456,10 +2686,10 @@
       <c r="C55" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D55" s="41"/>
-      <c r="E55" s="41"/>
-    </row>
-    <row r="56" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D55" s="49"/>
+      <c r="E55" s="49"/>
+    </row>
+    <row r="56" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A56" s="8" t="s">
         <v>89</v>
       </c>
@@ -2469,10 +2699,10 @@
       <c r="C56" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D56" s="41"/>
-      <c r="E56" s="41"/>
-    </row>
-    <row r="57" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D56" s="49"/>
+      <c r="E56" s="49"/>
+    </row>
+    <row r="57" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A57" s="8" t="s">
         <v>90</v>
       </c>
@@ -2482,10 +2712,10 @@
       <c r="C57" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-    </row>
-    <row r="58" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D57" s="49"/>
+      <c r="E57" s="49"/>
+    </row>
+    <row r="58" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A58" s="8" t="s">
         <v>91</v>
       </c>
@@ -2495,10 +2725,10 @@
       <c r="C58" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D58" s="41"/>
-      <c r="E58" s="41"/>
-    </row>
-    <row r="59" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D58" s="49"/>
+      <c r="E58" s="49"/>
+    </row>
+    <row r="59" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A59" s="8" t="s">
         <v>92</v>
       </c>
@@ -2508,10 +2738,10 @@
       <c r="C59" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D59" s="41"/>
-      <c r="E59" s="41"/>
-    </row>
-    <row r="60" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D59" s="49"/>
+      <c r="E59" s="49"/>
+    </row>
+    <row r="60" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A60" s="8" t="s">
         <v>93</v>
       </c>
@@ -2521,10 +2751,10 @@
       <c r="C60" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D60" s="41"/>
-      <c r="E60" s="41"/>
-    </row>
-    <row r="61" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D60" s="49"/>
+      <c r="E60" s="49"/>
+    </row>
+    <row r="61" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A61" s="8" t="s">
         <v>94</v>
       </c>
@@ -2534,10 +2764,10 @@
       <c r="C61" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D61" s="41"/>
-      <c r="E61" s="41"/>
-    </row>
-    <row r="62" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D61" s="49"/>
+      <c r="E61" s="49"/>
+    </row>
+    <row r="62" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A62" s="8" t="s">
         <v>95</v>
       </c>
@@ -2547,10 +2777,10 @@
       <c r="C62" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D62" s="41"/>
-      <c r="E62" s="41"/>
-    </row>
-    <row r="63" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D62" s="49"/>
+      <c r="E62" s="49"/>
+    </row>
+    <row r="63" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A63" s="8" t="s">
         <v>96</v>
       </c>
@@ -2560,10 +2790,10 @@
       <c r="C63" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D63" s="41"/>
-      <c r="E63" s="41"/>
-    </row>
-    <row r="64" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D63" s="49"/>
+      <c r="E63" s="49"/>
+    </row>
+    <row r="64" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A64" s="8" t="s">
         <v>97</v>
       </c>
@@ -2573,10 +2803,10 @@
       <c r="C64" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D64" s="41"/>
-      <c r="E64" s="41"/>
-    </row>
-    <row r="65" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D64" s="49"/>
+      <c r="E64" s="49"/>
+    </row>
+    <row r="65" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A65" s="11" t="s">
         <v>98</v>
       </c>
@@ -2586,12 +2816,12 @@
       <c r="C65" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="46" t="s">
+      <c r="D65" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="E65" s="46"/>
-    </row>
-    <row r="66" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E65" s="48"/>
+    </row>
+    <row r="66" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A66" s="11" t="s">
         <v>100</v>
       </c>
@@ -2601,12 +2831,12 @@
       <c r="C66" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D66" s="46" t="s">
+      <c r="D66" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="E66" s="46"/>
-    </row>
-    <row r="67" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E66" s="48"/>
+    </row>
+    <row r="67" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A67" s="11" t="s">
         <v>101</v>
       </c>
@@ -2616,12 +2846,12 @@
       <c r="C67" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D67" s="46" t="s">
+      <c r="D67" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="E67" s="46"/>
-    </row>
-    <row r="68" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E67" s="48"/>
+    </row>
+    <row r="68" spans="1:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A68" s="11" t="s">
         <v>102</v>
       </c>
@@ -2631,18 +2861,29 @@
       <c r="C68" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D68" s="46" t="s">
+      <c r="D68" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="E68" s="46"/>
+      <c r="E68" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A7:A11"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="A12:A16"/>
@@ -2659,41 +2900,591 @@
     <mergeCell ref="D61:E61"/>
     <mergeCell ref="D62:E62"/>
     <mergeCell ref="D63:E63"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="D37:E37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D175D2D-D7FE-4E32-BBA1-C84370195703}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64E7F13B-DF1D-4278-9622-0955E2C9E290}">
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="30.73046875" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="21.46484375" style="13" customWidth="1"/>
+    <col min="4" max="4" width="24.86328125" style="13" customWidth="1"/>
+    <col min="5" max="5" width="33.19921875" customWidth="1"/>
+    <col min="6" max="6" width="30.86328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="34" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="35"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3" s="43"/>
+      <c r="B3" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="35" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="43"/>
+      <c r="B4" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="35"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5" s="43"/>
+      <c r="B5" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="35"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6" s="43"/>
+      <c r="B6" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="35"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7" s="42" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="66"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" s="42"/>
+      <c r="B8" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="64"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A9" s="42"/>
+      <c r="B9" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="64"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" s="42"/>
+      <c r="B10" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="64"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11" s="42"/>
+      <c r="B11" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="65"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12" s="47" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="E12" t="s">
+        <v>161</v>
+      </c>
+      <c r="F12" s="66" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13" s="47"/>
+      <c r="B13" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" s="64"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14" s="47"/>
+      <c r="B14" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="F14" s="64"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15" s="47"/>
+      <c r="B15" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="64"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16" s="47"/>
+      <c r="B16" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="65"/>
+    </row>
+    <row r="17" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A17" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="63" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18" s="42" t="s">
+        <v>154</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="35"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" s="42"/>
+      <c r="B19" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="35"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20" s="42"/>
+      <c r="B20" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="35"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21" s="42"/>
+      <c r="B21" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="35"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22" s="50" t="s">
+        <v>149</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="35"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23" s="51"/>
+      <c r="B23" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="35"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="35"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A25" s="52" t="s">
+        <v>145</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="35"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A26" s="53"/>
+      <c r="B26" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="35"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A27" s="42" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="35"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A28" s="42"/>
+      <c r="B28" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="35"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A29" s="42"/>
+      <c r="B29" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="35"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A30" s="42"/>
+      <c r="B30" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="35"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A31" s="41" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" s="59" t="s">
+        <v>151</v>
+      </c>
+      <c r="C31" s="60"/>
+      <c r="D31" s="60"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="62"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A32" s="55" t="s">
+        <v>146</v>
+      </c>
+      <c r="B32" s="56"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="57"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="58"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C36"/>
+      <c r="D36"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C37"/>
+      <c r="D37"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C38"/>
+      <c r="D38"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C39"/>
+      <c r="D39"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C40"/>
+      <c r="D40"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C41"/>
+      <c r="D41"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C42"/>
+      <c r="D42"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C43"/>
+      <c r="D43"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C44"/>
+      <c r="D44"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C45"/>
+      <c r="D45"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C46"/>
+      <c r="D46"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C47"/>
+      <c r="D47"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="C48"/>
+      <c r="D48"/>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C49"/>
+      <c r="D49"/>
+    </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C50"/>
+      <c r="D50"/>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C51"/>
+      <c r="D51"/>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C52"/>
+      <c r="D52"/>
+    </row>
+    <row r="53" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C53"/>
+      <c r="D53"/>
+    </row>
+    <row r="54" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C54"/>
+      <c r="D54"/>
+    </row>
+    <row r="55" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C55"/>
+      <c r="D55"/>
+    </row>
+    <row r="56" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C56"/>
+      <c r="D56"/>
+    </row>
+    <row r="57" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C57"/>
+      <c r="D57"/>
+    </row>
+    <row r="58" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C58"/>
+      <c r="D58"/>
+    </row>
+    <row r="59" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C59"/>
+      <c r="D59"/>
+    </row>
+    <row r="60" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C60"/>
+      <c r="D60"/>
+    </row>
+    <row r="61" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C61"/>
+      <c r="D61"/>
+    </row>
+    <row r="62" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C62"/>
+      <c r="D62"/>
+    </row>
+    <row r="63" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C63"/>
+      <c r="D63"/>
+    </row>
+    <row r="64" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C64"/>
+      <c r="D64"/>
+    </row>
+    <row r="65" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C65"/>
+      <c r="D65"/>
+    </row>
+    <row r="66" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C66"/>
+      <c r="D66"/>
+    </row>
+    <row r="67" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C67"/>
+      <c r="D67"/>
+    </row>
+    <row r="68" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C68"/>
+      <c r="D68"/>
+    </row>
+    <row r="69" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C69"/>
+      <c r="D69"/>
+    </row>
+    <row r="70" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C70"/>
+      <c r="D70"/>
+    </row>
+    <row r="71" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C71"/>
+      <c r="D71"/>
+    </row>
+    <row r="72" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C72"/>
+      <c r="D72"/>
+    </row>
+    <row r="73" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C73"/>
+      <c r="D73"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="F12:F16"/>
+    <mergeCell ref="F7:F11"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A25:A26"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589B7773-EF81-4C25-9FB6-3256651D0E56}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D175D2D-D7FE-4E32-BBA1-C84370195703}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2701,11 +3492,31 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{589B7773-EF81-4C25-9FB6-3256651D0E56}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E15759AA-6F0D-4BB4-BC60-0CB52BC58382}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBD4978-CE40-4957-9D6C-78848C677960}">
   <dimension ref="A24:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="s">
         <v>128</v>
       </c>
@@ -2716,7 +3527,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>131</v>
       </c>
@@ -2727,7 +3538,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>133</v>
       </c>
@@ -2738,7 +3549,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>110</v>
       </c>
@@ -2749,7 +3560,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>137</v>
       </c>
@@ -2760,7 +3571,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -2771,7 +3582,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>140</v>
       </c>

</xml_diff>